<commit_message>
Add Lec 43 and 42 files of OOPs
</commit_message>
<xml_diff>
--- a/Complete DSA Notes/AlgoForge Zero-to-Hero DSA Sheet.xlsx
+++ b/Complete DSA Notes/AlgoForge Zero-to-Hero DSA Sheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\DSA\Complete DSA Notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F560D2AE-1F5A-4C05-BDCF-4A9C1663DDBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99405DE6-B372-43A4-83B1-47398631F0E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1165" uniqueCount="1059">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1177" uniqueCount="1059">
   <si>
     <t xml:space="preserve">DSA Sheet by AlgoForge </t>
   </si>
@@ -4187,8 +4187,8 @@
     </row>
     <row r="50" spans="1:4" ht="13.2">
       <c r="A50" s="6"/>
-      <c r="B50" s="7" t="b">
-        <v>0</v>
+      <c r="B50" s="7" t="s">
+        <v>1056</v>
       </c>
       <c r="C50" s="6" t="s">
         <v>74</v>
@@ -4199,8 +4199,8 @@
     </row>
     <row r="51" spans="1:4" ht="13.2">
       <c r="A51" s="6"/>
-      <c r="B51" s="7" t="b">
-        <v>0</v>
+      <c r="B51" s="7" t="s">
+        <v>1056</v>
       </c>
       <c r="C51" s="6" t="s">
         <v>76</v>
@@ -4211,8 +4211,8 @@
     </row>
     <row r="52" spans="1:4" ht="13.2">
       <c r="A52" s="6"/>
-      <c r="B52" s="7" t="b">
-        <v>0</v>
+      <c r="B52" s="7" t="s">
+        <v>1056</v>
       </c>
       <c r="C52" s="6" t="s">
         <v>78</v>
@@ -4223,8 +4223,8 @@
     </row>
     <row r="53" spans="1:4" ht="13.2">
       <c r="A53" s="6"/>
-      <c r="B53" s="7" t="b">
-        <v>0</v>
+      <c r="B53" s="7" t="s">
+        <v>1056</v>
       </c>
       <c r="C53" s="6" t="s">
         <v>80</v>
@@ -4269,8 +4269,8 @@
     </row>
     <row r="58" spans="1:4" ht="13.2">
       <c r="A58" s="6"/>
-      <c r="B58" s="7" t="b">
-        <v>0</v>
+      <c r="B58" s="7" t="s">
+        <v>1056</v>
       </c>
       <c r="C58" s="6" t="s">
         <v>87</v>
@@ -4278,8 +4278,8 @@
     </row>
     <row r="59" spans="1:4" ht="13.2">
       <c r="A59" s="6"/>
-      <c r="B59" s="7" t="b">
-        <v>0</v>
+      <c r="B59" s="7" t="s">
+        <v>1056</v>
       </c>
       <c r="C59" s="6" t="s">
         <v>88</v>
@@ -4290,8 +4290,8 @@
     </row>
     <row r="60" spans="1:4" ht="13.2">
       <c r="A60" s="6"/>
-      <c r="B60" s="7" t="b">
-        <v>0</v>
+      <c r="B60" s="7" t="s">
+        <v>1056</v>
       </c>
       <c r="C60" s="6" t="s">
         <v>90</v>
@@ -4314,8 +4314,8 @@
     </row>
     <row r="62" spans="1:4" ht="13.2">
       <c r="A62" s="6"/>
-      <c r="B62" s="7" t="b">
-        <v>0</v>
+      <c r="B62" s="7" t="s">
+        <v>1056</v>
       </c>
       <c r="C62" s="6" t="s">
         <v>94</v>
@@ -4323,8 +4323,8 @@
     </row>
     <row r="63" spans="1:4" ht="13.2">
       <c r="A63" s="6"/>
-      <c r="B63" s="7" t="b">
-        <v>0</v>
+      <c r="B63" s="7" t="s">
+        <v>1056</v>
       </c>
       <c r="C63" s="6" t="s">
         <v>95</v>
@@ -4335,8 +4335,8 @@
     </row>
     <row r="64" spans="1:4" ht="13.2">
       <c r="A64" s="6"/>
-      <c r="B64" s="7" t="b">
-        <v>0</v>
+      <c r="B64" s="7" t="s">
+        <v>1056</v>
       </c>
       <c r="C64" s="6" t="s">
         <v>97</v>
@@ -4347,8 +4347,8 @@
     </row>
     <row r="65" spans="1:4" ht="13.2">
       <c r="A65" s="6"/>
-      <c r="B65" s="7" t="b">
-        <v>0</v>
+      <c r="B65" s="7" t="s">
+        <v>1056</v>
       </c>
       <c r="C65" s="6" t="s">
         <v>99</v>
@@ -4356,8 +4356,8 @@
     </row>
     <row r="66" spans="1:4" ht="13.2">
       <c r="A66" s="6"/>
-      <c r="B66" s="7" t="b">
-        <v>0</v>
+      <c r="B66" s="7" t="s">
+        <v>1056</v>
       </c>
       <c r="C66" s="6" t="s">
         <v>100</v>

</xml_diff>

<commit_message>
Add lec 44 notes and singly linked list code
</commit_message>
<xml_diff>
--- a/Complete DSA Notes/AlgoForge Zero-to-Hero DSA Sheet.xlsx
+++ b/Complete DSA Notes/AlgoForge Zero-to-Hero DSA Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\DSA\Complete DSA Notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99405DE6-B372-43A4-83B1-47398631F0E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{929B6255-186B-4978-835F-0BB3C1F2B549}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1177" uniqueCount="1059">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1182" uniqueCount="1059">
   <si>
     <t xml:space="preserve">DSA Sheet by AlgoForge </t>
   </si>
@@ -4257,8 +4257,8 @@
     </row>
     <row r="57" spans="1:4" ht="13.2">
       <c r="A57" s="6"/>
-      <c r="B57" s="7" t="b">
-        <v>0</v>
+      <c r="B57" s="7" t="s">
+        <v>1056</v>
       </c>
       <c r="C57" s="6" t="s">
         <v>85</v>
@@ -4392,8 +4392,8 @@
     </row>
     <row r="71" spans="1:4" ht="13.2">
       <c r="A71" s="6"/>
-      <c r="B71" s="7" t="b">
-        <v>0</v>
+      <c r="B71" s="7" t="s">
+        <v>1056</v>
       </c>
       <c r="C71" s="6" t="s">
         <v>104</v>
@@ -4404,8 +4404,8 @@
     </row>
     <row r="72" spans="1:4" ht="13.2">
       <c r="A72" s="6"/>
-      <c r="B72" s="7" t="b">
-        <v>0</v>
+      <c r="B72" s="7" t="s">
+        <v>1056</v>
       </c>
       <c r="C72" s="6" t="s">
         <v>106</v>
@@ -4416,8 +4416,8 @@
     </row>
     <row r="73" spans="1:4" ht="13.2">
       <c r="A73" s="6"/>
-      <c r="B73" s="7" t="b">
-        <v>0</v>
+      <c r="B73" s="7" t="s">
+        <v>1056</v>
       </c>
       <c r="C73" s="6" t="s">
         <v>108</v>
@@ -4428,8 +4428,8 @@
     </row>
     <row r="74" spans="1:4" ht="13.2">
       <c r="A74" s="6"/>
-      <c r="B74" s="7" t="b">
-        <v>0</v>
+      <c r="B74" s="7" t="s">
+        <v>1056</v>
       </c>
       <c r="C74" s="6" t="s">
         <v>110</v>

</xml_diff>

<commit_message>
Add Uplot lec 49 Codes
</commit_message>
<xml_diff>
--- a/Complete DSA Notes/AlgoForge Zero-to-Hero DSA Sheet.xlsx
+++ b/Complete DSA Notes/AlgoForge Zero-to-Hero DSA Sheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\DSA\Complete DSA Notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{929B6255-186B-4978-835F-0BB3C1F2B549}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0E585C9-930A-441C-9DEE-6BBC01F521A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1182" uniqueCount="1059">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1184" uniqueCount="1059">
   <si>
     <t xml:space="preserve">DSA Sheet by AlgoForge </t>
   </si>
@@ -3260,7 +3260,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="28">
+  <fonts count="29">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -3427,6 +3427,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -3451,10 +3458,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3483,8 +3491,10 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -4447,8 +4457,8 @@
     </row>
     <row r="77" spans="1:4" ht="13.2">
       <c r="A77" s="6"/>
-      <c r="B77" s="7" t="b">
-        <v>0</v>
+      <c r="B77" s="7" t="s">
+        <v>1056</v>
       </c>
       <c r="C77" s="6" t="s">
         <v>113</v>
@@ -5226,13 +5236,13 @@
     </row>
     <row r="160" spans="1:4" ht="13.2">
       <c r="A160" s="6"/>
-      <c r="B160" s="7" t="b">
-        <v>0</v>
+      <c r="B160" s="7" t="s">
+        <v>1056</v>
       </c>
       <c r="C160" s="6" t="s">
         <v>224</v>
       </c>
-      <c r="D160" s="4" t="s">
+      <c r="D160" s="28" t="s">
         <v>225</v>
       </c>
     </row>

</xml_diff>